<commit_message>
Expand related research references
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/related research/paper_references.xlsx
+++ b/related research/paper_references.xlsx
@@ -10,7 +10,7 @@
     <sheet name="References" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'References'!$A$1:$J$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'References'!$A$1:$K$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -152,19 +152,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PaperReferences" displayName="PaperReferences" ref="A1:J2" headerRowCount="1">
-  <autoFilter ref="A1:J2"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PaperReferences" displayName="PaperReferences" ref="A1:K8" headerRowCount="1">
+  <autoFilter ref="A1:K8"/>
+  <tableColumns count="11">
     <tableColumn id="1" name="Authors"/>
     <tableColumn id="2" name="Year"/>
     <tableColumn id="3" name="Title"/>
-    <tableColumn id="4" name="Journal"/>
-    <tableColumn id="5" name="Volume"/>
-    <tableColumn id="6" name="Issue"/>
-    <tableColumn id="7" name="Pages"/>
-    <tableColumn id="8" name="DOI"/>
-    <tableColumn id="9" name="Repository record"/>
-    <tableColumn id="10" name="PDF access"/>
+    <tableColumn id="4" name="Type"/>
+    <tableColumn id="5" name="Journal / Series"/>
+    <tableColumn id="6" name="Volume"/>
+    <tableColumn id="7" name="Issue"/>
+    <tableColumn id="8" name="Pages / Article"/>
+    <tableColumn id="9" name="DOI"/>
+    <tableColumn id="10" name="Source / Record"/>
+    <tableColumn id="11" name="PDF / Access note"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -459,22 +460,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
-    <col width="58" customWidth="1" min="9" max="9"/>
-    <col width="76" customWidth="1" min="10" max="10"/>
+    <col width="72" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="43" customWidth="1" min="9" max="9"/>
+    <col width="68" customWidth="1" min="10" max="10"/>
+    <col width="74" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Authors</t>
@@ -492,41 +494,46 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Journal / Series</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Volume</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Issue</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Pages</t>
-        </is>
-      </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Pages / Article</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Repository record</t>
-        </is>
-      </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>PDF access</t>
+          <t>Source / Record</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>PDF / Access note</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="45" customHeight="1">
+    <row r="2" ht="58" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Mariano M. Croce; Thien T. Nguyen; Steve Raymond; Lukas Schmid</t>
@@ -542,45 +549,353 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>Research article</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>Journal of Financial Economics</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="F2" s="2" t="n">
         <v>132</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="G2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>205–225</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>205-225</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jfineco.2018.11.010</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>https://iris.unibocconi.it/handle/11565/4012542</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>No authorized public PDF identified; the Bocconi repository lists the post-print as restricted access.</t>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Bocconi repository lists the post-print as restricted access; no authorized public PDF identified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="58" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Michal Szudejko</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Government Debt and the Returns to Innovation (Summary)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Research summary</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>CFA Digest</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>January 2020</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>https://rpc.cfainstitute.org/research/cfa-digest/2020/01/dig-v50-n1-1</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Public CFA Digest summary of Croce et al.; this is a summary, not a separate research paper.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Yi Huang; Marco Pagano; Ugo Panizza</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Local Crowding-Out in China</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Research article</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>The Journal of Finance</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>2855-2898</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/jofi.12966</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>https://academicnewsletter.sufe.edu.cn/info/359227</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>PDF not downloaded; source link provided.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Cristina Arellano; Yan Bai; Luigi Bocola</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Sovereign Default Risk and Firm Heterogeneity</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Staff report</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Federal Reserve Bank of Minneapolis Staff Report 547; NBER Working Paper 23314 (2017)</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21034/sr.547</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>https://minneapolisfed.org/research/staff-reports/sovereign-default-risk-and-firm-heterogeneity</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>PDF not downloaded; the linked Minneapolis Fed page is the staff-report record.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Margherita Bottero; Simone Lenzu; Filippo Mezzanotti</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Sovereign debt exposure and the bank lending channel: Impact on credit supply and the real economy</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Research article</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Journal of International Economics</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>126</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>103328</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jinteco.2020.103328</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>https://academicnewsletter.sufe.edu.cn/info/297406</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>PDF not downloaded; source link provided.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Laura Blattner; Luisa Farinha; Francisca Rebelo</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>When Losses Turn into Loans: The Cost of Weak Banks</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Research article</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>American Economic Review</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>113</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>1600-1641</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1257/aer.20190149</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>https://cefup-nipe-rank.eeg.uminho.pt/people/430/articles</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>PDF not downloaded; source link provided.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Alexander Chudik; Kamiar Mohaddes; M. Hashem Pesaran; Mehdi Raissi</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>2017</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Is There a Debt-Threshold Effect on Output Growth?</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Research article</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Review of Economics and Statistics</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>135-150</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1162/rest_a_00593</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.econ.cam.ac.uk/research/pub-abstracts?pub=1281</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>PDF not downloaded; DOI links to the journal record.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J2"/>
+  <autoFilter ref="A1:K8"/>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId13"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId14"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>